<commit_message>
Update ranking at 2026-03-02 13:50
</commit_message>
<xml_diff>
--- a/amazonranking_matome.xlsx
+++ b/amazonranking_matome.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1993"/>
+  <dimension ref="A1:K1994"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -103338,6 +103338,63 @@
         </is>
       </c>
     </row>
+    <row r="1994">
+      <c r="A1994" t="inlineStr">
+        <is>
+          <t>2026/03/02 22:00</t>
+        </is>
+      </c>
+      <c r="B1994" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C1994" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D1994" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E1994" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F1994" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G1994" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1994" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I1994" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J1994" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K1994" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update ranking at 2026-03-02 14:33
</commit_message>
<xml_diff>
--- a/amazonranking_matome.xlsx
+++ b/amazonranking_matome.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1994"/>
+  <dimension ref="A1:K1995"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -103395,6 +103395,63 @@
         </is>
       </c>
     </row>
+    <row r="1995">
+      <c r="A1995" t="inlineStr">
+        <is>
+          <t>2026/03/02 23:00</t>
+        </is>
+      </c>
+      <c r="B1995" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C1995" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D1995" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E1995" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F1995" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G1995" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1995" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I1995" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J1995" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K1995" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update ranking at 2026-03-02 15:29
</commit_message>
<xml_diff>
--- a/amazonranking_matome.xlsx
+++ b/amazonranking_matome.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1995"/>
+  <dimension ref="A1:K1996"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -103452,6 +103452,63 @@
         </is>
       </c>
     </row>
+    <row r="1996">
+      <c r="A1996" t="inlineStr">
+        <is>
+          <t>2026/03/03 00:00</t>
+        </is>
+      </c>
+      <c r="B1996" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C1996" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D1996" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E1996" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F1996" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G1996" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1996" t="inlineStr">
+        <is>
+          <t>2,552位Audibleオーディオブック</t>
+        </is>
+      </c>
+      <c r="I1996" t="inlineStr">
+        <is>
+          <t>1位PR・広報</t>
+        </is>
+      </c>
+      <c r="J1996" t="inlineStr">
+        <is>
+          <t>1,364位ビジネス・経済 (本)</t>
+        </is>
+      </c>
+      <c r="K1996" t="inlineStr">
+        <is>
+          <t>3,128位ノンフィクション (本)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update ranking at 2026-03-02 16:28
</commit_message>
<xml_diff>
--- a/amazonranking_matome.xlsx
+++ b/amazonranking_matome.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1996"/>
+  <dimension ref="A1:K1997"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -103509,6 +103509,63 @@
         </is>
       </c>
     </row>
+    <row r="1997">
+      <c r="A1997" t="inlineStr">
+        <is>
+          <t>2026/03/03 01:00</t>
+        </is>
+      </c>
+      <c r="B1997" t="inlineStr">
+        <is>
+          <t>9,248位本</t>
+        </is>
+      </c>
+      <c r="C1997" t="inlineStr">
+        <is>
+          <t>27位広告・宣伝 (本)</t>
+        </is>
+      </c>
+      <c r="D1997" t="inlineStr">
+        <is>
+          <t>33位商業デザイン</t>
+        </is>
+      </c>
+      <c r="E1997" t="inlineStr">
+        <is>
+          <t>611位ビジネス実用本</t>
+        </is>
+      </c>
+      <c r="F1997" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G1997" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1997" t="inlineStr">
+        <is>
+          <t>2,552位Audibleオーディオブック</t>
+        </is>
+      </c>
+      <c r="I1997" t="inlineStr">
+        <is>
+          <t>1位PR・広報</t>
+        </is>
+      </c>
+      <c r="J1997" t="inlineStr">
+        <is>
+          <t>1,364位ビジネス・経済 (本)</t>
+        </is>
+      </c>
+      <c r="K1997" t="inlineStr">
+        <is>
+          <t>3,128位ノンフィクション (本)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update ranking at 2026-03-02 17:34
</commit_message>
<xml_diff>
--- a/amazonranking_matome.xlsx
+++ b/amazonranking_matome.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1997"/>
+  <dimension ref="A1:K1998"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -103566,6 +103566,63 @@
         </is>
       </c>
     </row>
+    <row r="1998">
+      <c r="A1998" t="inlineStr">
+        <is>
+          <t>2026/03/03 02:00</t>
+        </is>
+      </c>
+      <c r="B1998" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C1998" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D1998" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E1998" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F1998" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G1998" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1998" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I1998" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J1998" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K1998" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update ranking at 2026-03-02 18:29
</commit_message>
<xml_diff>
--- a/amazonranking_matome.xlsx
+++ b/amazonranking_matome.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1998"/>
+  <dimension ref="A1:K1999"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -103623,6 +103623,63 @@
         </is>
       </c>
     </row>
+    <row r="1999">
+      <c r="A1999" t="inlineStr">
+        <is>
+          <t>2026/03/03 03:00</t>
+        </is>
+      </c>
+      <c r="B1999" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C1999" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D1999" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E1999" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F1999" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G1999" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1999" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I1999" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J1999" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K1999" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update ranking at 2026-03-02 19:28
</commit_message>
<xml_diff>
--- a/amazonranking_matome.xlsx
+++ b/amazonranking_matome.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1999"/>
+  <dimension ref="A1:K2000"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -103680,6 +103680,63 @@
         </is>
       </c>
     </row>
+    <row r="2000">
+      <c r="A2000" t="inlineStr">
+        <is>
+          <t>2026/03/03 04:00</t>
+        </is>
+      </c>
+      <c r="B2000" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C2000" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D2000" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E2000" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F2000" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G2000" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H2000" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I2000" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J2000" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K2000" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update ranking at 2026-03-02 20:21
</commit_message>
<xml_diff>
--- a/amazonranking_matome.xlsx
+++ b/amazonranking_matome.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2000"/>
+  <dimension ref="A1:K2001"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -103737,6 +103737,63 @@
         </is>
       </c>
     </row>
+    <row r="2001">
+      <c r="A2001" t="inlineStr">
+        <is>
+          <t>2026/03/03 05:00</t>
+        </is>
+      </c>
+      <c r="B2001" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C2001" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D2001" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E2001" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F2001" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G2001" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H2001" t="inlineStr">
+        <is>
+          <t>2,727位Audibleオーディオブック</t>
+        </is>
+      </c>
+      <c r="I2001" t="inlineStr">
+        <is>
+          <t>1位PR・広報</t>
+        </is>
+      </c>
+      <c r="J2001" t="inlineStr">
+        <is>
+          <t>1,368位ビジネス・経済 (本)</t>
+        </is>
+      </c>
+      <c r="K2001" t="inlineStr">
+        <is>
+          <t>3,120位ノンフィクション (本)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update ranking at 2026-03-02 21:22
</commit_message>
<xml_diff>
--- a/amazonranking_matome.xlsx
+++ b/amazonranking_matome.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2001"/>
+  <dimension ref="A1:K2002"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -103794,6 +103794,63 @@
         </is>
       </c>
     </row>
+    <row r="2002">
+      <c r="A2002" t="inlineStr">
+        <is>
+          <t>2026/03/03 06:00</t>
+        </is>
+      </c>
+      <c r="B2002" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C2002" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D2002" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E2002" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F2002" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G2002" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H2002" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I2002" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J2002" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K2002" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update ranking at 2026-03-02 22:16
</commit_message>
<xml_diff>
--- a/amazonranking_matome.xlsx
+++ b/amazonranking_matome.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2002"/>
+  <dimension ref="A1:K2003"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -103851,6 +103851,63 @@
         </is>
       </c>
     </row>
+    <row r="2003">
+      <c r="A2003" t="inlineStr">
+        <is>
+          <t>2026/03/03 07:00</t>
+        </is>
+      </c>
+      <c r="B2003" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C2003" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D2003" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E2003" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F2003" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G2003" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H2003" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I2003" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J2003" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K2003" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update ranking at 2026-03-02 23:13
</commit_message>
<xml_diff>
--- a/amazonranking_matome.xlsx
+++ b/amazonranking_matome.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2003"/>
+  <dimension ref="A1:K2004"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -103908,6 +103908,63 @@
         </is>
       </c>
     </row>
+    <row r="2004">
+      <c r="A2004" t="inlineStr">
+        <is>
+          <t>2026/03/03 08:00</t>
+        </is>
+      </c>
+      <c r="B2004" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C2004" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D2004" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E2004" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F2004" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G2004" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H2004" t="inlineStr">
+        <is>
+          <t>2,727位Audibleオーディオブック</t>
+        </is>
+      </c>
+      <c r="I2004" t="inlineStr">
+        <is>
+          <t>1位PR・広報</t>
+        </is>
+      </c>
+      <c r="J2004" t="inlineStr">
+        <is>
+          <t>1,368位ビジネス・経済 (本)</t>
+        </is>
+      </c>
+      <c r="K2004" t="inlineStr">
+        <is>
+          <t>3,120位ノンフィクション (本)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update ranking at 2026-03-03 01:00
</commit_message>
<xml_diff>
--- a/amazonranking_matome.xlsx
+++ b/amazonranking_matome.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2004"/>
+  <dimension ref="A1:K2005"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -103965,6 +103965,63 @@
         </is>
       </c>
     </row>
+    <row r="2005">
+      <c r="A2005" t="inlineStr">
+        <is>
+          <t>2026/03/03 10:00</t>
+        </is>
+      </c>
+      <c r="B2005" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C2005" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D2005" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E2005" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F2005" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G2005" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H2005" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I2005" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J2005" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K2005" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update ranking at 2026-03-03 04:02
</commit_message>
<xml_diff>
--- a/amazonranking_matome.xlsx
+++ b/amazonranking_matome.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2005"/>
+  <dimension ref="A1:K2006"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -104022,6 +104022,63 @@
         </is>
       </c>
     </row>
+    <row r="2006">
+      <c r="A2006" t="inlineStr">
+        <is>
+          <t>2026/03/03 13:00</t>
+        </is>
+      </c>
+      <c r="B2006" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C2006" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D2006" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E2006" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F2006" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G2006" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H2006" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I2006" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J2006" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K2006" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update ranking at 2026-03-03 05:39
</commit_message>
<xml_diff>
--- a/amazonranking_matome.xlsx
+++ b/amazonranking_matome.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2006"/>
+  <dimension ref="A1:K2007"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -104079,6 +104079,63 @@
         </is>
       </c>
     </row>
+    <row r="2007">
+      <c r="A2007" t="inlineStr">
+        <is>
+          <t>2026/03/03 14:00</t>
+        </is>
+      </c>
+      <c r="B2007" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C2007" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D2007" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E2007" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F2007" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G2007" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H2007" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I2007" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J2007" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K2007" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update ranking at 2026-03-03 06:34
</commit_message>
<xml_diff>
--- a/amazonranking_matome.xlsx
+++ b/amazonranking_matome.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2007"/>
+  <dimension ref="A1:K2008"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -104136,6 +104136,63 @@
         </is>
       </c>
     </row>
+    <row r="2008">
+      <c r="A2008" t="inlineStr">
+        <is>
+          <t>2026/03/03 15:00</t>
+        </is>
+      </c>
+      <c r="B2008" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C2008" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D2008" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E2008" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F2008" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G2008" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H2008" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I2008" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J2008" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K2008" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update ranking at 2026-03-03 07:33
</commit_message>
<xml_diff>
--- a/amazonranking_matome.xlsx
+++ b/amazonranking_matome.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2008"/>
+  <dimension ref="A1:K2009"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -104193,6 +104193,63 @@
         </is>
       </c>
     </row>
+    <row r="2009">
+      <c r="A2009" t="inlineStr">
+        <is>
+          <t>2026/03/03 16:00</t>
+        </is>
+      </c>
+      <c r="B2009" t="inlineStr">
+        <is>
+          <t>10,396位本</t>
+        </is>
+      </c>
+      <c r="C2009" t="inlineStr">
+        <is>
+          <t>33位広告・宣伝 (本)</t>
+        </is>
+      </c>
+      <c r="D2009" t="inlineStr">
+        <is>
+          <t>36位商業デザイン</t>
+        </is>
+      </c>
+      <c r="E2009" t="inlineStr">
+        <is>
+          <t>700位ビジネス実用本</t>
+        </is>
+      </c>
+      <c r="F2009" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G2009" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H2009" t="inlineStr">
+        <is>
+          <t>3,068位Audibleオーディオブック</t>
+        </is>
+      </c>
+      <c r="I2009" t="inlineStr">
+        <is>
+          <t>1位PR・広報</t>
+        </is>
+      </c>
+      <c r="J2009" t="inlineStr">
+        <is>
+          <t>1,573位ビジネス・経済 (本)</t>
+        </is>
+      </c>
+      <c r="K2009" t="inlineStr">
+        <is>
+          <t>3,715位ノンフィクション (本)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update ranking at 2026-03-03 08:26
</commit_message>
<xml_diff>
--- a/amazonranking_matome.xlsx
+++ b/amazonranking_matome.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2009"/>
+  <dimension ref="A1:K2010"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -104250,6 +104250,63 @@
         </is>
       </c>
     </row>
+    <row r="2010">
+      <c r="A2010" t="inlineStr">
+        <is>
+          <t>2026/03/03 17:00</t>
+        </is>
+      </c>
+      <c r="B2010" t="inlineStr">
+        <is>
+          <t>10,396位本</t>
+        </is>
+      </c>
+      <c r="C2010" t="inlineStr">
+        <is>
+          <t>33位広告・宣伝 (本)</t>
+        </is>
+      </c>
+      <c r="D2010" t="inlineStr">
+        <is>
+          <t>36位商業デザイン</t>
+        </is>
+      </c>
+      <c r="E2010" t="inlineStr">
+        <is>
+          <t>700位ビジネス実用本</t>
+        </is>
+      </c>
+      <c r="F2010" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G2010" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H2010" t="inlineStr">
+        <is>
+          <t>3,068位Audibleオーディオブック</t>
+        </is>
+      </c>
+      <c r="I2010" t="inlineStr">
+        <is>
+          <t>1位PR・広報</t>
+        </is>
+      </c>
+      <c r="J2010" t="inlineStr">
+        <is>
+          <t>1,573位ビジネス・経済 (本)</t>
+        </is>
+      </c>
+      <c r="K2010" t="inlineStr">
+        <is>
+          <t>3,715位ノンフィクション (本)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update ranking at 2026-03-03 09:29
</commit_message>
<xml_diff>
--- a/amazonranking_matome.xlsx
+++ b/amazonranking_matome.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2010"/>
+  <dimension ref="A1:K2011"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -104307,6 +104307,63 @@
         </is>
       </c>
     </row>
+    <row r="2011">
+      <c r="A2011" t="inlineStr">
+        <is>
+          <t>2026/03/03 18:00</t>
+        </is>
+      </c>
+      <c r="B2011" t="inlineStr">
+        <is>
+          <t>10,394位本</t>
+        </is>
+      </c>
+      <c r="C2011" t="inlineStr">
+        <is>
+          <t>33位広告・宣伝 (本)</t>
+        </is>
+      </c>
+      <c r="D2011" t="inlineStr">
+        <is>
+          <t>36位商業デザイン</t>
+        </is>
+      </c>
+      <c r="E2011" t="inlineStr">
+        <is>
+          <t>700位ビジネス実用本</t>
+        </is>
+      </c>
+      <c r="F2011" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G2011" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H2011" t="inlineStr">
+        <is>
+          <t>3,068位Audibleオーディオブック</t>
+        </is>
+      </c>
+      <c r="I2011" t="inlineStr">
+        <is>
+          <t>1位PR・広報</t>
+        </is>
+      </c>
+      <c r="J2011" t="inlineStr">
+        <is>
+          <t>1,573位ビジネス・経済 (本)</t>
+        </is>
+      </c>
+      <c r="K2011" t="inlineStr">
+        <is>
+          <t>3,715位ノンフィクション (本)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update ranking at 2026-03-03 10:26
</commit_message>
<xml_diff>
--- a/amazonranking_matome.xlsx
+++ b/amazonranking_matome.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2011"/>
+  <dimension ref="A1:K2012"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -104364,6 +104364,63 @@
         </is>
       </c>
     </row>
+    <row r="2012">
+      <c r="A2012" t="inlineStr">
+        <is>
+          <t>2026/03/03 19:00</t>
+        </is>
+      </c>
+      <c r="B2012" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C2012" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D2012" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E2012" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F2012" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G2012" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H2012" t="inlineStr">
+        <is>
+          <t>3,068位Audibleオーディオブック</t>
+        </is>
+      </c>
+      <c r="I2012" t="inlineStr">
+        <is>
+          <t>1位PR・広報</t>
+        </is>
+      </c>
+      <c r="J2012" t="inlineStr">
+        <is>
+          <t>1,573位ビジネス・経済 (本)</t>
+        </is>
+      </c>
+      <c r="K2012" t="inlineStr">
+        <is>
+          <t>3,715位ノンフィクション (本)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update ranking at 2026-03-03 11:22
</commit_message>
<xml_diff>
--- a/amazonranking_matome.xlsx
+++ b/amazonranking_matome.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2012"/>
+  <dimension ref="A1:K2013"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -104421,6 +104421,63 @@
         </is>
       </c>
     </row>
+    <row r="2013">
+      <c r="A2013" t="inlineStr">
+        <is>
+          <t>2026/03/03 20:00</t>
+        </is>
+      </c>
+      <c r="B2013" t="inlineStr">
+        <is>
+          <t>10,394位本</t>
+        </is>
+      </c>
+      <c r="C2013" t="inlineStr">
+        <is>
+          <t>33位広告・宣伝 (本)</t>
+        </is>
+      </c>
+      <c r="D2013" t="inlineStr">
+        <is>
+          <t>36位商業デザイン</t>
+        </is>
+      </c>
+      <c r="E2013" t="inlineStr">
+        <is>
+          <t>700位ビジネス実用本</t>
+        </is>
+      </c>
+      <c r="F2013" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G2013" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H2013" t="inlineStr">
+        <is>
+          <t>3,068位Audibleオーディオブック</t>
+        </is>
+      </c>
+      <c r="I2013" t="inlineStr">
+        <is>
+          <t>1位PR・広報</t>
+        </is>
+      </c>
+      <c r="J2013" t="inlineStr">
+        <is>
+          <t>1,573位ビジネス・経済 (本)</t>
+        </is>
+      </c>
+      <c r="K2013" t="inlineStr">
+        <is>
+          <t>3,715位ノンフィクション (本)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update ranking at 2026-03-03 12:28
</commit_message>
<xml_diff>
--- a/amazonranking_matome.xlsx
+++ b/amazonranking_matome.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2013"/>
+  <dimension ref="A1:K2014"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -104478,6 +104478,63 @@
         </is>
       </c>
     </row>
+    <row r="2014">
+      <c r="A2014" t="inlineStr">
+        <is>
+          <t>2026/03/03 21:00</t>
+        </is>
+      </c>
+      <c r="B2014" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C2014" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D2014" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E2014" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F2014" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G2014" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H2014" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I2014" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J2014" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K2014" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update ranking at 2026-03-03 13:49
</commit_message>
<xml_diff>
--- a/amazonranking_matome.xlsx
+++ b/amazonranking_matome.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2014"/>
+  <dimension ref="A1:K2015"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -104535,6 +104535,63 @@
         </is>
       </c>
     </row>
+    <row r="2015">
+      <c r="A2015" t="inlineStr">
+        <is>
+          <t>2026/03/03 22:00</t>
+        </is>
+      </c>
+      <c r="B2015" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C2015" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D2015" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E2015" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F2015" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G2015" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H2015" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I2015" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J2015" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K2015" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update ranking at 2026-03-03 14:34
</commit_message>
<xml_diff>
--- a/amazonranking_matome.xlsx
+++ b/amazonranking_matome.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2015"/>
+  <dimension ref="A1:K2016"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -104592,6 +104592,63 @@
         </is>
       </c>
     </row>
+    <row r="2016">
+      <c r="A2016" t="inlineStr">
+        <is>
+          <t>2026/03/03 23:00</t>
+        </is>
+      </c>
+      <c r="B2016" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C2016" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D2016" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E2016" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F2016" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G2016" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H2016" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I2016" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J2016" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K2016" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update ranking at 2026-03-03 15:35
</commit_message>
<xml_diff>
--- a/amazonranking_matome.xlsx
+++ b/amazonranking_matome.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2016"/>
+  <dimension ref="A1:K2017"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -104649,6 +104649,63 @@
         </is>
       </c>
     </row>
+    <row r="2017">
+      <c r="A2017" t="inlineStr">
+        <is>
+          <t>2026/03/04 00:00</t>
+        </is>
+      </c>
+      <c r="B2017" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C2017" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D2017" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E2017" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F2017" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G2017" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H2017" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I2017" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J2017" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K2017" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update ranking at 2026-03-03 16:31
</commit_message>
<xml_diff>
--- a/amazonranking_matome.xlsx
+++ b/amazonranking_matome.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2017"/>
+  <dimension ref="A1:K2018"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -104706,6 +104706,63 @@
         </is>
       </c>
     </row>
+    <row r="2018">
+      <c r="A2018" t="inlineStr">
+        <is>
+          <t>2026/03/04 01:00</t>
+        </is>
+      </c>
+      <c r="B2018" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C2018" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D2018" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E2018" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F2018" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G2018" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H2018" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I2018" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J2018" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K2018" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update ranking at 2026-03-03 17:33
</commit_message>
<xml_diff>
--- a/amazonranking_matome.xlsx
+++ b/amazonranking_matome.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2018"/>
+  <dimension ref="A1:K2019"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -104763,6 +104763,63 @@
         </is>
       </c>
     </row>
+    <row r="2019">
+      <c r="A2019" t="inlineStr">
+        <is>
+          <t>2026/03/04 02:00</t>
+        </is>
+      </c>
+      <c r="B2019" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C2019" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D2019" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E2019" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F2019" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G2019" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H2019" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I2019" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J2019" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K2019" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update ranking at 2026-03-03 18:31
</commit_message>
<xml_diff>
--- a/amazonranking_matome.xlsx
+++ b/amazonranking_matome.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2019"/>
+  <dimension ref="A1:K2020"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -104820,6 +104820,63 @@
         </is>
       </c>
     </row>
+    <row r="2020">
+      <c r="A2020" t="inlineStr">
+        <is>
+          <t>2026/03/04 03:00</t>
+        </is>
+      </c>
+      <c r="B2020" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C2020" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D2020" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E2020" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F2020" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G2020" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H2020" t="inlineStr">
+        <is>
+          <t>3,389位Audibleオーディオブック</t>
+        </is>
+      </c>
+      <c r="I2020" t="inlineStr">
+        <is>
+          <t>1位PR・広報</t>
+        </is>
+      </c>
+      <c r="J2020" t="inlineStr">
+        <is>
+          <t>2,397位ビジネス・経済 (本)</t>
+        </is>
+      </c>
+      <c r="K2020" t="inlineStr">
+        <is>
+          <t>5,636位ノンフィクション (本)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update ranking at 2026-03-03 19:32
</commit_message>
<xml_diff>
--- a/amazonranking_matome.xlsx
+++ b/amazonranking_matome.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2020"/>
+  <dimension ref="A1:K2021"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -104877,6 +104877,63 @@
         </is>
       </c>
     </row>
+    <row r="2021">
+      <c r="A2021" t="inlineStr">
+        <is>
+          <t>2026/03/04 04:00</t>
+        </is>
+      </c>
+      <c r="B2021" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C2021" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D2021" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E2021" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F2021" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G2021" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H2021" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I2021" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J2021" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K2021" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update ranking at 2026-03-03 20:19
</commit_message>
<xml_diff>
--- a/amazonranking_matome.xlsx
+++ b/amazonranking_matome.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2021"/>
+  <dimension ref="A1:K2022"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -104934,6 +104934,63 @@
         </is>
       </c>
     </row>
+    <row r="2022">
+      <c r="A2022" t="inlineStr">
+        <is>
+          <t>2026/03/04 05:00</t>
+        </is>
+      </c>
+      <c r="B2022" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C2022" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D2022" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E2022" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F2022" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G2022" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H2022" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I2022" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J2022" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K2022" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update ranking at 2026-03-03 21:22
</commit_message>
<xml_diff>
--- a/amazonranking_matome.xlsx
+++ b/amazonranking_matome.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2022"/>
+  <dimension ref="A1:K2023"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -104991,6 +104991,63 @@
         </is>
       </c>
     </row>
+    <row r="2023">
+      <c r="A2023" t="inlineStr">
+        <is>
+          <t>2026/03/04 06:00</t>
+        </is>
+      </c>
+      <c r="B2023" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C2023" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D2023" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E2023" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F2023" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G2023" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H2023" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I2023" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J2023" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K2023" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update ranking at 2026-03-03 22:15
</commit_message>
<xml_diff>
--- a/amazonranking_matome.xlsx
+++ b/amazonranking_matome.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2023"/>
+  <dimension ref="A1:K2024"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -105048,6 +105048,63 @@
         </is>
       </c>
     </row>
+    <row r="2024">
+      <c r="A2024" t="inlineStr">
+        <is>
+          <t>2026/03/04 07:00</t>
+        </is>
+      </c>
+      <c r="B2024" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C2024" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D2024" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E2024" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F2024" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G2024" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H2024" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I2024" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J2024" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K2024" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update ranking at 2026-03-03 23:14
</commit_message>
<xml_diff>
--- a/amazonranking_matome.xlsx
+++ b/amazonranking_matome.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2024"/>
+  <dimension ref="A1:K2025"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -105105,6 +105105,63 @@
         </is>
       </c>
     </row>
+    <row r="2025">
+      <c r="A2025" t="inlineStr">
+        <is>
+          <t>2026/03/04 08:00</t>
+        </is>
+      </c>
+      <c r="B2025" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C2025" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D2025" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E2025" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F2025" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G2025" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H2025" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I2025" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J2025" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K2025" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update ranking at 2026-03-04 00:57
</commit_message>
<xml_diff>
--- a/amazonranking_matome.xlsx
+++ b/amazonranking_matome.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2025"/>
+  <dimension ref="A1:K2026"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -105162,6 +105162,63 @@
         </is>
       </c>
     </row>
+    <row r="2026">
+      <c r="A2026" t="inlineStr">
+        <is>
+          <t>2026/03/04 09:00</t>
+        </is>
+      </c>
+      <c r="B2026" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C2026" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D2026" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E2026" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F2026" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G2026" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H2026" t="inlineStr">
+        <is>
+          <t>3,390位Audibleオーディオブック</t>
+        </is>
+      </c>
+      <c r="I2026" t="inlineStr">
+        <is>
+          <t>1位PR・広報</t>
+        </is>
+      </c>
+      <c r="J2026" t="inlineStr">
+        <is>
+          <t>2,397位ビジネス・経済 (本)</t>
+        </is>
+      </c>
+      <c r="K2026" t="inlineStr">
+        <is>
+          <t>5,636位ノンフィクション (本)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update ranking at 2026-03-04 03:22
</commit_message>
<xml_diff>
--- a/amazonranking_matome.xlsx
+++ b/amazonranking_matome.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2026"/>
+  <dimension ref="A1:K2027"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -105219,6 +105219,63 @@
         </is>
       </c>
     </row>
+    <row r="2027">
+      <c r="A2027" t="inlineStr">
+        <is>
+          <t>2026/03/04 12:00</t>
+        </is>
+      </c>
+      <c r="B2027" t="inlineStr">
+        <is>
+          <t>21,263位本</t>
+        </is>
+      </c>
+      <c r="C2027" t="inlineStr">
+        <is>
+          <t>59位広告・宣伝 (本)</t>
+        </is>
+      </c>
+      <c r="D2027" t="inlineStr">
+        <is>
+          <t>68位商業デザイン</t>
+        </is>
+      </c>
+      <c r="E2027" t="inlineStr">
+        <is>
+          <t>1,269位ビジネス実用本</t>
+        </is>
+      </c>
+      <c r="F2027" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G2027" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H2027" t="inlineStr">
+        <is>
+          <t>3,565位Audibleオーディオブック</t>
+        </is>
+      </c>
+      <c r="I2027" t="inlineStr">
+        <is>
+          <t>1位PR・広報</t>
+        </is>
+      </c>
+      <c r="J2027" t="inlineStr">
+        <is>
+          <t>2,905位ビジネス・経済 (本)</t>
+        </is>
+      </c>
+      <c r="K2027" t="inlineStr">
+        <is>
+          <t>6,963位ノンフィクション (本)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update ranking at 2026-03-04 05:02
</commit_message>
<xml_diff>
--- a/amazonranking_matome.xlsx
+++ b/amazonranking_matome.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2027"/>
+  <dimension ref="A1:K2028"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -105276,6 +105276,63 @@
         </is>
       </c>
     </row>
+    <row r="2028">
+      <c r="A2028" t="inlineStr">
+        <is>
+          <t>2026/03/04 14:00</t>
+        </is>
+      </c>
+      <c r="B2028" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C2028" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D2028" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E2028" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F2028" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G2028" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H2028" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I2028" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J2028" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K2028" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update ranking at 2026-03-04 06:31
</commit_message>
<xml_diff>
--- a/amazonranking_matome.xlsx
+++ b/amazonranking_matome.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2028"/>
+  <dimension ref="A1:K2029"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -105333,6 +105333,63 @@
         </is>
       </c>
     </row>
+    <row r="2029">
+      <c r="A2029" t="inlineStr">
+        <is>
+          <t>2026/03/04 15:00</t>
+        </is>
+      </c>
+      <c r="B2029" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C2029" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D2029" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E2029" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F2029" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G2029" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H2029" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I2029" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J2029" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K2029" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update ranking at 2026-03-04 07:29
</commit_message>
<xml_diff>
--- a/amazonranking_matome.xlsx
+++ b/amazonranking_matome.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2029"/>
+  <dimension ref="A1:K2030"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -105390,6 +105390,63 @@
         </is>
       </c>
     </row>
+    <row r="2030">
+      <c r="A2030" t="inlineStr">
+        <is>
+          <t>2026/03/04 16:00</t>
+        </is>
+      </c>
+      <c r="B2030" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C2030" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D2030" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E2030" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F2030" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G2030" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H2030" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I2030" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J2030" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K2030" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update ranking at 2026-03-04 08:23
</commit_message>
<xml_diff>
--- a/amazonranking_matome.xlsx
+++ b/amazonranking_matome.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2030"/>
+  <dimension ref="A1:K2031"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -105447,6 +105447,63 @@
         </is>
       </c>
     </row>
+    <row r="2031">
+      <c r="A2031" t="inlineStr">
+        <is>
+          <t>2026/03/04 17:00</t>
+        </is>
+      </c>
+      <c r="B2031" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C2031" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D2031" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E2031" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F2031" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G2031" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H2031" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I2031" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J2031" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K2031" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update ranking at 2026-03-04 09:28
</commit_message>
<xml_diff>
--- a/amazonranking_matome.xlsx
+++ b/amazonranking_matome.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2031"/>
+  <dimension ref="A1:K2032"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -105504,6 +105504,63 @@
         </is>
       </c>
     </row>
+    <row r="2032">
+      <c r="A2032" t="inlineStr">
+        <is>
+          <t>2026/03/04 18:00</t>
+        </is>
+      </c>
+      <c r="B2032" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C2032" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D2032" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E2032" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F2032" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G2032" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H2032" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I2032" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J2032" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K2032" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update ranking at 2026-03-04 10:23
</commit_message>
<xml_diff>
--- a/amazonranking_matome.xlsx
+++ b/amazonranking_matome.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2032"/>
+  <dimension ref="A1:K2033"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -105561,6 +105561,63 @@
         </is>
       </c>
     </row>
+    <row r="2033">
+      <c r="A2033" t="inlineStr">
+        <is>
+          <t>2026/03/04 19:00</t>
+        </is>
+      </c>
+      <c r="B2033" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C2033" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D2033" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E2033" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F2033" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G2033" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H2033" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I2033" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J2033" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K2033" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update ranking at 2026-03-04 11:20
</commit_message>
<xml_diff>
--- a/amazonranking_matome.xlsx
+++ b/amazonranking_matome.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2033"/>
+  <dimension ref="A1:K2034"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -105618,6 +105618,63 @@
         </is>
       </c>
     </row>
+    <row r="2034">
+      <c r="A2034" t="inlineStr">
+        <is>
+          <t>2026/03/04 20:00</t>
+        </is>
+      </c>
+      <c r="B2034" t="inlineStr">
+        <is>
+          <t>21,549位本</t>
+        </is>
+      </c>
+      <c r="C2034" t="inlineStr">
+        <is>
+          <t>61位広告・宣伝 (本)</t>
+        </is>
+      </c>
+      <c r="D2034" t="inlineStr">
+        <is>
+          <t>75位商業デザイン</t>
+        </is>
+      </c>
+      <c r="E2034" t="inlineStr">
+        <is>
+          <t>1,290位ビジネス実用本</t>
+        </is>
+      </c>
+      <c r="F2034" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G2034" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H2034" t="inlineStr">
+        <is>
+          <t>3,696位Audibleオーディオブック</t>
+        </is>
+      </c>
+      <c r="I2034" t="inlineStr">
+        <is>
+          <t>1位PR・広報</t>
+        </is>
+      </c>
+      <c r="J2034" t="inlineStr">
+        <is>
+          <t>2,943位ビジネス・経済 (本)</t>
+        </is>
+      </c>
+      <c r="K2034" t="inlineStr">
+        <is>
+          <t>7,093位ノンフィクション (本)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update ranking at 2026-03-04 12:27
</commit_message>
<xml_diff>
--- a/amazonranking_matome.xlsx
+++ b/amazonranking_matome.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2034"/>
+  <dimension ref="A1:K2035"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -105675,6 +105675,63 @@
         </is>
       </c>
     </row>
+    <row r="2035">
+      <c r="A2035" t="inlineStr">
+        <is>
+          <t>2026/03/04 21:00</t>
+        </is>
+      </c>
+      <c r="B2035" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C2035" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D2035" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E2035" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F2035" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G2035" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H2035" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I2035" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J2035" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K2035" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update ranking at 2026-03-04 13:46
</commit_message>
<xml_diff>
--- a/amazonranking_matome.xlsx
+++ b/amazonranking_matome.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2035"/>
+  <dimension ref="A1:K2036"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -105732,6 +105732,63 @@
         </is>
       </c>
     </row>
+    <row r="2036">
+      <c r="A2036" t="inlineStr">
+        <is>
+          <t>2026/03/04 22:00</t>
+        </is>
+      </c>
+      <c r="B2036" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C2036" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D2036" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E2036" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F2036" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G2036" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H2036" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I2036" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J2036" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K2036" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update ranking at 2026-03-04 14:29
</commit_message>
<xml_diff>
--- a/amazonranking_matome.xlsx
+++ b/amazonranking_matome.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2036"/>
+  <dimension ref="A1:K2037"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -105789,6 +105789,63 @@
         </is>
       </c>
     </row>
+    <row r="2037">
+      <c r="A2037" t="inlineStr">
+        <is>
+          <t>2026/03/04 23:00</t>
+        </is>
+      </c>
+      <c r="B2037" t="inlineStr">
+        <is>
+          <t>12,641位本</t>
+        </is>
+      </c>
+      <c r="C2037" t="inlineStr">
+        <is>
+          <t>39位広告・宣伝 (本)</t>
+        </is>
+      </c>
+      <c r="D2037" t="inlineStr">
+        <is>
+          <t>41位商業デザイン</t>
+        </is>
+      </c>
+      <c r="E2037" t="inlineStr">
+        <is>
+          <t>863位ビジネス実用本</t>
+        </is>
+      </c>
+      <c r="F2037" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G2037" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H2037" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I2037" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J2037" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K2037" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update ranking at 2026-03-04 15:27
</commit_message>
<xml_diff>
--- a/amazonranking_matome.xlsx
+++ b/amazonranking_matome.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2037"/>
+  <dimension ref="A1:K2038"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -105846,6 +105846,63 @@
         </is>
       </c>
     </row>
+    <row r="2038">
+      <c r="A2038" t="inlineStr">
+        <is>
+          <t>2026/03/05 00:00</t>
+        </is>
+      </c>
+      <c r="B2038" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C2038" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D2038" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E2038" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F2038" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G2038" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H2038" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I2038" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J2038" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K2038" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update ranking at 2026-03-04 16:28
</commit_message>
<xml_diff>
--- a/amazonranking_matome.xlsx
+++ b/amazonranking_matome.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2038"/>
+  <dimension ref="A1:K2039"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -105903,6 +105903,63 @@
         </is>
       </c>
     </row>
+    <row r="2039">
+      <c r="A2039" t="inlineStr">
+        <is>
+          <t>2026/03/05 01:00</t>
+        </is>
+      </c>
+      <c r="B2039" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C2039" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D2039" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E2039" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F2039" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G2039" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H2039" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I2039" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J2039" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K2039" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update ranking at 2026-03-04 17:29
</commit_message>
<xml_diff>
--- a/amazonranking_matome.xlsx
+++ b/amazonranking_matome.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2039"/>
+  <dimension ref="A1:K2040"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -105960,6 +105960,63 @@
         </is>
       </c>
     </row>
+    <row r="2040">
+      <c r="A2040" t="inlineStr">
+        <is>
+          <t>2026/03/05 02:00</t>
+        </is>
+      </c>
+      <c r="B2040" t="inlineStr">
+        <is>
+          <t>12,641位本</t>
+        </is>
+      </c>
+      <c r="C2040" t="inlineStr">
+        <is>
+          <t>39位広告・宣伝 (本)</t>
+        </is>
+      </c>
+      <c r="D2040" t="inlineStr">
+        <is>
+          <t>39位商業デザイン</t>
+        </is>
+      </c>
+      <c r="E2040" t="inlineStr">
+        <is>
+          <t>863位ビジネス実用本</t>
+        </is>
+      </c>
+      <c r="F2040" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G2040" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H2040" t="inlineStr">
+        <is>
+          <t>3,806位Audibleオーディオブック</t>
+        </is>
+      </c>
+      <c r="I2040" t="inlineStr">
+        <is>
+          <t>1位PR・広報</t>
+        </is>
+      </c>
+      <c r="J2040" t="inlineStr">
+        <is>
+          <t>1,938位ビジネス・経済 (本)</t>
+        </is>
+      </c>
+      <c r="K2040" t="inlineStr">
+        <is>
+          <t>4,505位ノンフィクション (本)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update ranking at 2026-03-04 18:30
</commit_message>
<xml_diff>
--- a/amazonranking_matome.xlsx
+++ b/amazonranking_matome.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2040"/>
+  <dimension ref="A1:K2041"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -106017,6 +106017,63 @@
         </is>
       </c>
     </row>
+    <row r="2041">
+      <c r="A2041" t="inlineStr">
+        <is>
+          <t>2026/03/05 03:00</t>
+        </is>
+      </c>
+      <c r="B2041" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C2041" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D2041" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E2041" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F2041" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G2041" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H2041" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I2041" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J2041" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K2041" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update ranking at 2026-03-04 19:29
</commit_message>
<xml_diff>
--- a/amazonranking_matome.xlsx
+++ b/amazonranking_matome.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2041"/>
+  <dimension ref="A1:K2042"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -106074,6 +106074,63 @@
         </is>
       </c>
     </row>
+    <row r="2042">
+      <c r="A2042" t="inlineStr">
+        <is>
+          <t>2026/03/05 04:00</t>
+        </is>
+      </c>
+      <c r="B2042" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C2042" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D2042" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E2042" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F2042" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G2042" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H2042" t="inlineStr">
+        <is>
+          <t>3,806位Audibleオーディオブック</t>
+        </is>
+      </c>
+      <c r="I2042" t="inlineStr">
+        <is>
+          <t>1位PR・広報</t>
+        </is>
+      </c>
+      <c r="J2042" t="inlineStr">
+        <is>
+          <t>1,938位ビジネス・経済 (本)</t>
+        </is>
+      </c>
+      <c r="K2042" t="inlineStr">
+        <is>
+          <t>4,505位ノンフィクション (本)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update ranking at 2026-03-04 20:20
</commit_message>
<xml_diff>
--- a/amazonranking_matome.xlsx
+++ b/amazonranking_matome.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2042"/>
+  <dimension ref="A1:K2043"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -106131,6 +106131,63 @@
         </is>
       </c>
     </row>
+    <row r="2043">
+      <c r="A2043" t="inlineStr">
+        <is>
+          <t>2026/03/05 05:00</t>
+        </is>
+      </c>
+      <c r="B2043" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C2043" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D2043" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E2043" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F2043" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G2043" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H2043" t="inlineStr">
+        <is>
+          <t>3,925位Audibleオーディオブック</t>
+        </is>
+      </c>
+      <c r="I2043" t="inlineStr">
+        <is>
+          <t>1位PR・広報</t>
+        </is>
+      </c>
+      <c r="J2043" t="inlineStr">
+        <is>
+          <t>2,435位ビジネス・経済 (本)</t>
+        </is>
+      </c>
+      <c r="K2043" t="inlineStr">
+        <is>
+          <t>5,662位ノンフィクション (本)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update ranking at 2026-03-04 21:21
</commit_message>
<xml_diff>
--- a/amazonranking_matome.xlsx
+++ b/amazonranking_matome.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2043"/>
+  <dimension ref="A1:K2044"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -106188,6 +106188,63 @@
         </is>
       </c>
     </row>
+    <row r="2044">
+      <c r="A2044" t="inlineStr">
+        <is>
+          <t>2026/03/05 06:00</t>
+        </is>
+      </c>
+      <c r="B2044" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C2044" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D2044" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E2044" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F2044" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G2044" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H2044" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I2044" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J2044" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K2044" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update ranking at 2026-03-04 22:18
</commit_message>
<xml_diff>
--- a/amazonranking_matome.xlsx
+++ b/amazonranking_matome.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2044"/>
+  <dimension ref="A1:K2045"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -106245,6 +106245,63 @@
         </is>
       </c>
     </row>
+    <row r="2045">
+      <c r="A2045" t="inlineStr">
+        <is>
+          <t>2026/03/05 07:00</t>
+        </is>
+      </c>
+      <c r="B2045" t="inlineStr">
+        <is>
+          <t>16,404位本</t>
+        </is>
+      </c>
+      <c r="C2045" t="inlineStr">
+        <is>
+          <t>50位商業デザイン</t>
+        </is>
+      </c>
+      <c r="D2045" t="inlineStr">
+        <is>
+          <t>52位広告・宣伝 (本)</t>
+        </is>
+      </c>
+      <c r="E2045" t="inlineStr">
+        <is>
+          <t>1,090位ビジネス実用本</t>
+        </is>
+      </c>
+      <c r="F2045" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G2045" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H2045" t="inlineStr">
+        <is>
+          <t>3,926位Audibleオーディオブック</t>
+        </is>
+      </c>
+      <c r="I2045" t="inlineStr">
+        <is>
+          <t>1位PR・広報</t>
+        </is>
+      </c>
+      <c r="J2045" t="inlineStr">
+        <is>
+          <t>2,435位ビジネス・経済 (本)</t>
+        </is>
+      </c>
+      <c r="K2045" t="inlineStr">
+        <is>
+          <t>5,662位ノンフィクション (本)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update ranking at 2026-03-04 23:18
</commit_message>
<xml_diff>
--- a/amazonranking_matome.xlsx
+++ b/amazonranking_matome.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2045"/>
+  <dimension ref="A1:K2046"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -106302,6 +106302,63 @@
         </is>
       </c>
     </row>
+    <row r="2046">
+      <c r="A2046" t="inlineStr">
+        <is>
+          <t>2026/03/05 08:00</t>
+        </is>
+      </c>
+      <c r="B2046" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C2046" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D2046" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E2046" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F2046" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G2046" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H2046" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I2046" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J2046" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K2046" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update ranking at 2026-03-05 00:59
</commit_message>
<xml_diff>
--- a/amazonranking_matome.xlsx
+++ b/amazonranking_matome.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2046"/>
+  <dimension ref="A1:K2047"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -106359,6 +106359,63 @@
         </is>
       </c>
     </row>
+    <row r="2047">
+      <c r="A2047" t="inlineStr">
+        <is>
+          <t>2026/03/05 09:00</t>
+        </is>
+      </c>
+      <c r="B2047" t="inlineStr">
+        <is>
+          <t>16,404位本</t>
+        </is>
+      </c>
+      <c r="C2047" t="inlineStr">
+        <is>
+          <t>50位商業デザイン</t>
+        </is>
+      </c>
+      <c r="D2047" t="inlineStr">
+        <is>
+          <t>52位広告・宣伝 (本)</t>
+        </is>
+      </c>
+      <c r="E2047" t="inlineStr">
+        <is>
+          <t>1,090位ビジネス実用本</t>
+        </is>
+      </c>
+      <c r="F2047" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G2047" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H2047" t="inlineStr">
+        <is>
+          <t>3,926位Audibleオーディオブック</t>
+        </is>
+      </c>
+      <c r="I2047" t="inlineStr">
+        <is>
+          <t>1位PR・広報</t>
+        </is>
+      </c>
+      <c r="J2047" t="inlineStr">
+        <is>
+          <t>2,435位ビジネス・経済 (本)</t>
+        </is>
+      </c>
+      <c r="K2047" t="inlineStr">
+        <is>
+          <t>5,662位ノンフィクション (本)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update ranking at 2026-03-05 03:28
</commit_message>
<xml_diff>
--- a/amazonranking_matome.xlsx
+++ b/amazonranking_matome.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2047"/>
+  <dimension ref="A1:K2048"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -106416,6 +106416,63 @@
         </is>
       </c>
     </row>
+    <row r="2048">
+      <c r="A2048" t="inlineStr">
+        <is>
+          <t>2026/03/05 12:00</t>
+        </is>
+      </c>
+      <c r="B2048" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C2048" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D2048" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E2048" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F2048" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G2048" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H2048" t="inlineStr">
+        <is>
+          <t>4,134位Audibleオーディオブック</t>
+        </is>
+      </c>
+      <c r="I2048" t="inlineStr">
+        <is>
+          <t>1位PR・広報</t>
+        </is>
+      </c>
+      <c r="J2048" t="inlineStr">
+        <is>
+          <t>1,496位ビジネス・経済 (本)</t>
+        </is>
+      </c>
+      <c r="K2048" t="inlineStr">
+        <is>
+          <t>3,468位ノンフィクション (本)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update ranking at 2026-03-05 05:07
</commit_message>
<xml_diff>
--- a/amazonranking_matome.xlsx
+++ b/amazonranking_matome.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2048"/>
+  <dimension ref="A1:K2049"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -106473,6 +106473,63 @@
         </is>
       </c>
     </row>
+    <row r="2049">
+      <c r="A2049" t="inlineStr">
+        <is>
+          <t>2026/03/05 14:00</t>
+        </is>
+      </c>
+      <c r="B2049" t="inlineStr">
+        <is>
+          <t>9,472位本</t>
+        </is>
+      </c>
+      <c r="C2049" t="inlineStr">
+        <is>
+          <t>29位広告・宣伝 (本)</t>
+        </is>
+      </c>
+      <c r="D2049" t="inlineStr">
+        <is>
+          <t>29位商業デザイン</t>
+        </is>
+      </c>
+      <c r="E2049" t="inlineStr">
+        <is>
+          <t>653位ビジネス実用本</t>
+        </is>
+      </c>
+      <c r="F2049" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G2049" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H2049" t="inlineStr">
+        <is>
+          <t>4,134位Audibleオーディオブック</t>
+        </is>
+      </c>
+      <c r="I2049" t="inlineStr">
+        <is>
+          <t>1位PR・広報</t>
+        </is>
+      </c>
+      <c r="J2049" t="inlineStr">
+        <is>
+          <t>1,498位ビジネス・経済 (本)</t>
+        </is>
+      </c>
+      <c r="K2049" t="inlineStr">
+        <is>
+          <t>3,468位ノンフィクション (本)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update ranking at 2026-03-05 06:34
</commit_message>
<xml_diff>
--- a/amazonranking_matome.xlsx
+++ b/amazonranking_matome.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2049"/>
+  <dimension ref="A1:K2050"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -106530,6 +106530,63 @@
         </is>
       </c>
     </row>
+    <row r="2050">
+      <c r="A2050" t="inlineStr">
+        <is>
+          <t>2026/03/05 15:00</t>
+        </is>
+      </c>
+      <c r="B2050" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C2050" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D2050" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E2050" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F2050" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G2050" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H2050" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I2050" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J2050" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K2050" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update ranking at 2026-03-05 07:33
</commit_message>
<xml_diff>
--- a/amazonranking_matome.xlsx
+++ b/amazonranking_matome.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2050"/>
+  <dimension ref="A1:K2051"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -106587,6 +106587,63 @@
         </is>
       </c>
     </row>
+    <row r="2051">
+      <c r="A2051" t="inlineStr">
+        <is>
+          <t>2026/03/05 16:00</t>
+        </is>
+      </c>
+      <c r="B2051" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C2051" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D2051" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E2051" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F2051" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G2051" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H2051" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I2051" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J2051" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K2051" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update ranking at 2026-03-05 08:25
</commit_message>
<xml_diff>
--- a/amazonranking_matome.xlsx
+++ b/amazonranking_matome.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2051"/>
+  <dimension ref="A1:K2052"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -106644,6 +106644,63 @@
         </is>
       </c>
     </row>
+    <row r="2052">
+      <c r="A2052" t="inlineStr">
+        <is>
+          <t>2026/03/05 17:00</t>
+        </is>
+      </c>
+      <c r="B2052" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C2052" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D2052" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E2052" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F2052" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G2052" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H2052" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I2052" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J2052" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K2052" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update ranking at 2026-03-05 09:30
</commit_message>
<xml_diff>
--- a/amazonranking_matome.xlsx
+++ b/amazonranking_matome.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2052"/>
+  <dimension ref="A1:K2053"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -106701,6 +106701,63 @@
         </is>
       </c>
     </row>
+    <row r="2053">
+      <c r="A2053" t="inlineStr">
+        <is>
+          <t>2026/03/05 18:00</t>
+        </is>
+      </c>
+      <c r="B2053" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C2053" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D2053" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E2053" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F2053" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G2053" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H2053" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I2053" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J2053" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K2053" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update ranking at 2026-03-05 10:26
</commit_message>
<xml_diff>
--- a/amazonranking_matome.xlsx
+++ b/amazonranking_matome.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2053"/>
+  <dimension ref="A1:K2054"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -106758,6 +106758,63 @@
         </is>
       </c>
     </row>
+    <row r="2054">
+      <c r="A2054" t="inlineStr">
+        <is>
+          <t>2026/03/05 19:00</t>
+        </is>
+      </c>
+      <c r="B2054" t="inlineStr">
+        <is>
+          <t>10,251位本</t>
+        </is>
+      </c>
+      <c r="C2054" t="inlineStr">
+        <is>
+          <t>31位商業デザイン</t>
+        </is>
+      </c>
+      <c r="D2054" t="inlineStr">
+        <is>
+          <t>32位広告・宣伝 (本)</t>
+        </is>
+      </c>
+      <c r="E2054" t="inlineStr">
+        <is>
+          <t>701位ビジネス実用本</t>
+        </is>
+      </c>
+      <c r="F2054" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G2054" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H2054" t="inlineStr">
+        <is>
+          <t>4,311位Audibleオーディオブック</t>
+        </is>
+      </c>
+      <c r="I2054" t="inlineStr">
+        <is>
+          <t>1位PR・広報</t>
+        </is>
+      </c>
+      <c r="J2054" t="inlineStr">
+        <is>
+          <t>1,604位ビジネス・経済 (本)</t>
+        </is>
+      </c>
+      <c r="K2054" t="inlineStr">
+        <is>
+          <t>3,726位ノンフィクション (本)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update ranking at 2026-03-05 11:24
</commit_message>
<xml_diff>
--- a/amazonranking_matome.xlsx
+++ b/amazonranking_matome.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2054"/>
+  <dimension ref="A1:K2055"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -106815,6 +106815,63 @@
         </is>
       </c>
     </row>
+    <row r="2055">
+      <c r="A2055" t="inlineStr">
+        <is>
+          <t>2026/03/05 20:00</t>
+        </is>
+      </c>
+      <c r="B2055" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C2055" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D2055" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E2055" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F2055" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G2055" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H2055" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I2055" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J2055" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K2055" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update ranking at 2026-03-05 12:31
</commit_message>
<xml_diff>
--- a/amazonranking_matome.xlsx
+++ b/amazonranking_matome.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2055"/>
+  <dimension ref="A1:K2056"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -106872,6 +106872,63 @@
         </is>
       </c>
     </row>
+    <row r="2056">
+      <c r="A2056" t="inlineStr">
+        <is>
+          <t>2026/03/05 21:00</t>
+        </is>
+      </c>
+      <c r="B2056" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C2056" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D2056" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E2056" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F2056" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G2056" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H2056" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I2056" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J2056" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K2056" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>